<commit_message>
filter propertyType and budget + full output
</commit_message>
<xml_diff>
--- a/TripData.xlsx
+++ b/TripData.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t xml:space="preserve">Destination</t>
   </si>
@@ -34,10 +34,22 @@
     <t xml:space="preserve">Guests</t>
   </si>
   <si>
+    <t xml:space="preserve">PropertyType</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Budget</t>
+  </si>
+  <si>
     <t xml:space="preserve">Brasov</t>
   </si>
   <si>
+    <t xml:space="preserve">Hotels</t>
+  </si>
+  <si>
     <t xml:space="preserve">Milan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apartments</t>
   </si>
 </sst>
 </file>
@@ -126,15 +138,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -328,53 +340,71 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D1000"/>
+  <dimension ref="A1:F1000"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="15.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="15.11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="2" t="n">
+      <c r="A2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="3" t="n">
         <v>46157</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>46223</v>
       </c>
-      <c r="D2" s="1" t="n">
+      <c r="D2" s="2" t="n">
         <v>3</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="0" t="n">
+        <v>50000</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="2" t="n">
+      <c r="A3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="3" t="n">
         <v>46244</v>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="3" t="n">
         <v>46249</v>
       </c>
-      <c r="D3" s="1" t="n">
+      <c r="D3" s="2" t="n">
         <v>1</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="0" t="n">
+        <v>1000</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
added tripid and property type to booking sccraping
</commit_message>
<xml_diff>
--- a/TripData.xlsx
+++ b/TripData.xlsx
@@ -20,7 +20,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+  <si>
+    <t xml:space="preserve">TripId</t>
+  </si>
   <si>
     <t xml:space="preserve">Destination</t>
   </si>
@@ -340,7 +343,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F1000"/>
+  <dimension ref="A1:G1000"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.21"/>
@@ -348,7 +351,7 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
@@ -360,50 +363,59 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="3" t="n">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="3" t="n">
         <v>46157</v>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="D2" s="3" t="n">
         <v>46223</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="E2" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" s="0" t="n">
+      <c r="F2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="1" t="n">
         <v>50000</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="3" t="n">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="3" t="n">
         <v>46244</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="D3" s="3" t="n">
         <v>46249</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="E3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" s="0" t="n">
+      <c r="F3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="1" t="n">
         <v>1000</v>
       </c>
     </row>

</xml_diff>